<commit_message>
Complete table version 1
</commit_message>
<xml_diff>
--- a/data/manual/materials_prices.xlsx
+++ b/data/manual/materials_prices.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dpsich-my.sharepoint.com/personal/alvaro_hahn-menacho_psi_ch/Documents/Severin's work/3_Code/semesterproject/data/manual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="131" documentId="13_ncr:1_{D88AC83D-3D0E-48F6-B25A-3A931C8EAFD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3D7DC24-78F4-4671-BB8B-2374D4921DED}"/>
+  <xr:revisionPtr revIDLastSave="138" documentId="13_ncr:1_{D88AC83D-3D0E-48F6-B25A-3A931C8EAFD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31949691-E44D-420F-BA4F-560A928C2BB4}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="294">
   <si>
     <t>material_category</t>
   </si>
@@ -909,6 +909,12 @@
   </si>
   <si>
     <t>https://ecoquery.ecoinvent.org/3.11/cutoff/dataset/11094/exchanges</t>
+  </si>
+  <si>
+    <t>molybdenite</t>
+  </si>
+  <si>
+    <t>https://ecoquery.ecoinvent.org/3.11/cutoff/dataset/2695/exchanges</t>
   </si>
 </sst>
 </file>
@@ -973,7 +979,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -981,16 +987,13 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="11" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1304,7 +1307,7 @@
     <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="29.7109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="26.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.5703125" style="6" customWidth="1"/>
+    <col min="6" max="6" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -1346,7 +1349,7 @@
       <c r="E2" t="s">
         <v>185</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2">
         <v>0.84</v>
       </c>
       <c r="G2" s="2" t="s">
@@ -1369,7 +1372,7 @@
       <c r="E3" t="s">
         <v>186</v>
       </c>
-      <c r="F3" s="6">
+      <c r="F3">
         <v>9.0700000000000003E-2</v>
       </c>
       <c r="G3" s="2" t="s">
@@ -1392,7 +1395,7 @@
       <c r="E4" t="s">
         <v>190</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4">
         <v>2.9099999999999998E-3</v>
       </c>
       <c r="G4" s="2" t="s">
@@ -1415,7 +1418,7 @@
       <c r="E5" t="s">
         <v>191</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5">
         <v>0.92</v>
       </c>
       <c r="G5" s="2" t="s">
@@ -1438,7 +1441,7 @@
       <c r="E6" t="s">
         <v>194</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6">
         <v>0.88700000000000001</v>
       </c>
       <c r="G6" s="2" t="s">
@@ -1458,8 +1461,14 @@
       <c r="D7" t="s">
         <v>17</v>
       </c>
-      <c r="H7" t="s">
-        <v>195</v>
+      <c r="E7" t="s">
+        <v>292</v>
+      </c>
+      <c r="F7">
+        <v>5.84</v>
+      </c>
+      <c r="G7" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -1492,8 +1501,14 @@
       <c r="D9" t="s">
         <v>21</v>
       </c>
-      <c r="H9" t="s">
-        <v>195</v>
+      <c r="E9" t="s">
+        <v>190</v>
+      </c>
+      <c r="F9">
+        <v>2.9099999999999998E-3</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -1512,7 +1527,7 @@
       <c r="E10" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F10" s="3">
         <v>5.85</v>
       </c>
       <c r="G10" s="4" t="s">
@@ -1520,22 +1535,22 @@
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
+      <c r="A11" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="8" t="s">
         <v>25</v>
       </c>
       <c r="E11" t="s">
         <v>201</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11">
         <v>0.628</v>
       </c>
       <c r="G11" t="s">
@@ -1543,14 +1558,14 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="5"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
       <c r="E12" t="s">
         <v>199</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12">
         <v>1.72</v>
       </c>
       <c r="G12" t="s">
@@ -1590,7 +1605,7 @@
       <c r="E14" t="s">
         <v>207</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14">
         <v>8.3800000000000008</v>
       </c>
       <c r="G14" t="s">
@@ -1613,7 +1628,7 @@
       <c r="E15" s="3" t="s">
         <v>208</v>
       </c>
-      <c r="F15" s="7">
+      <c r="F15" s="3">
         <v>3.99</v>
       </c>
       <c r="G15" s="3" t="s">
@@ -1636,7 +1651,7 @@
       <c r="E16" t="s">
         <v>211</v>
       </c>
-      <c r="F16" s="6">
+      <c r="F16">
         <v>5.52</v>
       </c>
       <c r="G16" t="s">
@@ -1659,7 +1674,7 @@
       <c r="E17" s="3" t="s">
         <v>213</v>
       </c>
-      <c r="F17" s="7">
+      <c r="F17" s="3">
         <v>5.91E-2</v>
       </c>
       <c r="G17" s="3" t="s">
@@ -1682,7 +1697,7 @@
       <c r="E18" t="s">
         <v>214</v>
       </c>
-      <c r="F18" s="6">
+      <c r="F18">
         <v>4.9000000000000002E-2</v>
       </c>
       <c r="G18" t="s">
@@ -1756,7 +1771,7 @@
       <c r="E22" s="3" t="s">
         <v>218</v>
       </c>
-      <c r="F22" s="7">
+      <c r="F22" s="3">
         <v>0.21</v>
       </c>
       <c r="G22" s="3" t="s">
@@ -1779,7 +1794,7 @@
       <c r="E23" t="s">
         <v>219</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23">
         <v>1.6E-2</v>
       </c>
       <c r="G23" t="s">
@@ -1802,7 +1817,7 @@
       <c r="E24" t="s">
         <v>224</v>
       </c>
-      <c r="F24" s="6">
+      <c r="F24">
         <v>1.4E-2</v>
       </c>
       <c r="G24" t="s">
@@ -1825,7 +1840,7 @@
       <c r="E25" t="s">
         <v>227</v>
       </c>
-      <c r="F25" s="6">
+      <c r="F25">
         <v>7.5500000000000003E-3</v>
       </c>
       <c r="G25" t="s">
@@ -1848,7 +1863,7 @@
       <c r="E26" t="s">
         <v>220</v>
       </c>
-      <c r="F26" s="6">
+      <c r="F26">
         <v>0.13</v>
       </c>
       <c r="G26" t="s">
@@ -1871,7 +1886,7 @@
       <c r="E27" t="s">
         <v>218</v>
       </c>
-      <c r="F27" s="6">
+      <c r="F27">
         <v>0.21</v>
       </c>
       <c r="G27" t="s">
@@ -1896,22 +1911,22 @@
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="8" t="s">
         <v>65</v>
       </c>
       <c r="E29" t="s">
         <v>230</v>
       </c>
-      <c r="F29" s="6">
+      <c r="F29">
         <v>0.04</v>
       </c>
       <c r="G29" t="s">
@@ -1919,14 +1934,14 @@
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="5"/>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5"/>
-      <c r="D30" s="5"/>
+      <c r="A30" s="8"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
       <c r="E30" t="s">
         <v>231</v>
       </c>
-      <c r="F30" s="6">
+      <c r="F30">
         <v>4.53E-2</v>
       </c>
       <c r="G30" t="s">
@@ -1949,7 +1964,7 @@
       <c r="E31" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="F31" s="7">
+      <c r="F31" s="3">
         <v>0.84</v>
       </c>
       <c r="G31" s="3" t="s">
@@ -1972,7 +1987,7 @@
       <c r="E32" s="3" t="s">
         <v>235</v>
       </c>
-      <c r="F32" s="8">
+      <c r="F32" s="5">
         <v>21400</v>
       </c>
       <c r="G32" s="3" t="s">
@@ -2012,7 +2027,7 @@
       <c r="E34" s="3" t="s">
         <v>185</v>
       </c>
-      <c r="F34" s="7">
+      <c r="F34" s="3">
         <v>0.84</v>
       </c>
       <c r="G34" s="3" t="s">
@@ -2035,7 +2050,7 @@
       <c r="E35" t="s">
         <v>221</v>
       </c>
-      <c r="F35" s="6">
+      <c r="F35">
         <v>3.78E-2</v>
       </c>
       <c r="G35" t="s">
@@ -2058,7 +2073,7 @@
       <c r="E36" t="s">
         <v>238</v>
       </c>
-      <c r="F36" s="6">
+      <c r="F36">
         <v>0.17599999999999999</v>
       </c>
       <c r="G36" t="s">
@@ -2081,7 +2096,7 @@
       <c r="E37" t="s">
         <v>240</v>
       </c>
-      <c r="F37" s="6">
+      <c r="F37">
         <v>0.84599999999999997</v>
       </c>
       <c r="G37" t="s">
@@ -2104,7 +2119,7 @@
       <c r="E38" t="s">
         <v>222</v>
       </c>
-      <c r="F38" s="6">
+      <c r="F38">
         <v>1.1499999999999999</v>
       </c>
       <c r="G38" t="s">
@@ -2127,7 +2142,7 @@
       <c r="E39" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="F39" s="7">
+      <c r="F39" s="3">
         <v>1.24</v>
       </c>
       <c r="G39" s="3" t="s">
@@ -2150,7 +2165,7 @@
       <c r="E40" s="3" t="s">
         <v>245</v>
       </c>
-      <c r="F40" s="7">
+      <c r="F40" s="3">
         <v>11.2</v>
       </c>
       <c r="G40" s="3" t="s">
@@ -2173,7 +2188,7 @@
       <c r="E41" t="s">
         <v>247</v>
       </c>
-      <c r="F41" s="6">
+      <c r="F41">
         <v>432</v>
       </c>
       <c r="G41" t="s">
@@ -2213,7 +2228,7 @@
       <c r="E43" t="s">
         <v>249</v>
       </c>
-      <c r="F43" s="6">
+      <c r="F43">
         <v>9.3000000000000007</v>
       </c>
       <c r="G43" t="s">
@@ -2236,7 +2251,7 @@
       <c r="E44" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="F44" s="7">
+      <c r="F44" s="3">
         <v>5.85</v>
       </c>
       <c r="G44" s="4" t="s">
@@ -2259,7 +2274,7 @@
       <c r="E45" t="s">
         <v>194</v>
       </c>
-      <c r="F45" s="6">
+      <c r="F45">
         <v>0.88700000000000001</v>
       </c>
       <c r="G45" t="s">
@@ -2299,7 +2314,7 @@
       <c r="E47" t="s">
         <v>251</v>
       </c>
-      <c r="F47" s="9">
+      <c r="F47" s="6">
         <v>1360</v>
       </c>
       <c r="G47" t="s">
@@ -2339,7 +2354,7 @@
       <c r="E49" t="s">
         <v>253</v>
       </c>
-      <c r="F49" s="6">
+      <c r="F49">
         <v>1.1299999999999999E-2</v>
       </c>
       <c r="G49" t="s">
@@ -2362,7 +2377,7 @@
       <c r="E50" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="F50" s="7">
+      <c r="F50" s="3">
         <v>8.6900000000000005E-2</v>
       </c>
       <c r="G50" s="3" t="s">
@@ -2385,7 +2400,7 @@
       <c r="E51" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="F51" s="7">
+      <c r="F51" s="3">
         <v>8.6900000000000005E-2</v>
       </c>
       <c r="G51" s="3" t="s">
@@ -2408,7 +2423,7 @@
       <c r="E52" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="F52" s="7">
+      <c r="F52" s="3">
         <v>8.6900000000000005E-2</v>
       </c>
       <c r="G52" s="3" t="s">
@@ -2431,7 +2446,7 @@
       <c r="E53" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="F53" s="7">
+      <c r="F53" s="3">
         <v>8.6900000000000005E-2</v>
       </c>
       <c r="G53" s="3" t="s">
@@ -2454,7 +2469,7 @@
       <c r="E54" t="s">
         <v>257</v>
       </c>
-      <c r="F54" s="6">
+      <c r="F54">
         <v>4.0099999999999997E-2</v>
       </c>
       <c r="G54" t="s">
@@ -2477,7 +2492,7 @@
       <c r="E55" t="s">
         <v>255</v>
       </c>
-      <c r="F55" s="6">
+      <c r="F55">
         <v>8.6900000000000005E-2</v>
       </c>
       <c r="G55" t="s">
@@ -2500,7 +2515,7 @@
       <c r="E56" s="3" t="s">
         <v>259</v>
       </c>
-      <c r="F56" s="7">
+      <c r="F56" s="3">
         <v>0.99</v>
       </c>
       <c r="G56" s="3" t="s">
@@ -2523,7 +2538,7 @@
       <c r="E57" t="s">
         <v>261</v>
       </c>
-      <c r="F57" s="6">
+      <c r="F57">
         <v>0.88100000000000001</v>
       </c>
       <c r="G57" t="s">
@@ -2560,7 +2575,7 @@
       <c r="E59" t="s">
         <v>207</v>
       </c>
-      <c r="F59" s="6">
+      <c r="F59">
         <v>8.3800000000000008</v>
       </c>
       <c r="G59" t="s">
@@ -2568,22 +2583,22 @@
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="5" t="s">
+      <c r="A60" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="B60" s="5" t="s">
+      <c r="B60" s="8" t="s">
         <v>121</v>
       </c>
-      <c r="C60" s="5" t="s">
+      <c r="C60" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="D60" s="5" t="s">
+      <c r="D60" s="8" t="s">
         <v>129</v>
       </c>
       <c r="E60" t="s">
         <v>203</v>
       </c>
-      <c r="F60" s="6">
+      <c r="F60">
         <v>2.36</v>
       </c>
       <c r="G60" t="s">
@@ -2591,14 +2606,14 @@
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="5"/>
-      <c r="B61" s="5"/>
-      <c r="C61" s="5"/>
-      <c r="D61" s="5"/>
+      <c r="A61" s="8"/>
+      <c r="B61" s="8"/>
+      <c r="C61" s="8"/>
+      <c r="D61" s="8"/>
       <c r="E61" t="s">
         <v>205</v>
       </c>
-      <c r="F61" s="6">
+      <c r="F61">
         <v>22.5</v>
       </c>
       <c r="G61" t="s">
@@ -2621,7 +2636,7 @@
       <c r="E62" t="s">
         <v>264</v>
       </c>
-      <c r="F62" s="6">
+      <c r="F62">
         <v>445</v>
       </c>
       <c r="G62" t="s">
@@ -2644,7 +2659,7 @@
       <c r="E63" t="s">
         <v>265</v>
       </c>
-      <c r="F63" s="9">
+      <c r="F63" s="6">
         <v>35300</v>
       </c>
       <c r="G63" t="s">
@@ -2667,7 +2682,7 @@
       <c r="E64" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="F64" s="7">
+      <c r="F64" s="3">
         <v>5.52</v>
       </c>
       <c r="G64" s="3" t="s">
@@ -2690,7 +2705,7 @@
       <c r="E65" t="s">
         <v>194</v>
       </c>
-      <c r="F65" s="6">
+      <c r="F65">
         <v>2.13</v>
       </c>
       <c r="G65" t="s">
@@ -2713,7 +2728,7 @@
       <c r="E66" s="3" t="s">
         <v>278</v>
       </c>
-      <c r="F66" s="7">
+      <c r="F66" s="3">
         <v>12.5</v>
       </c>
       <c r="G66" s="3" t="s">
@@ -2736,7 +2751,7 @@
       <c r="E67" t="s">
         <v>266</v>
       </c>
-      <c r="F67" s="6">
+      <c r="F67">
         <v>1.64</v>
       </c>
       <c r="G67" t="s">
@@ -2756,10 +2771,10 @@
       <c r="D68" t="s">
         <v>144</v>
       </c>
-      <c r="E68" s="10" t="s">
+      <c r="E68" t="s">
         <v>267</v>
       </c>
-      <c r="F68" s="9">
+      <c r="F68" s="6">
         <v>24900</v>
       </c>
       <c r="G68" t="s">
@@ -2779,10 +2794,10 @@
       <c r="D69" t="s">
         <v>146</v>
       </c>
-      <c r="E69" s="10" t="s">
+      <c r="E69" t="s">
         <v>268</v>
       </c>
-      <c r="F69" s="9">
+      <c r="F69" s="6">
         <v>28100</v>
       </c>
       <c r="G69" t="s">
@@ -2802,10 +2817,10 @@
       <c r="D70" t="s">
         <v>148</v>
       </c>
-      <c r="E70" s="10" t="s">
+      <c r="E70" t="s">
         <v>269</v>
       </c>
-      <c r="F70" s="6">
+      <c r="F70">
         <v>32.1</v>
       </c>
       <c r="G70" t="s">
@@ -2825,10 +2840,10 @@
       <c r="D71" t="s">
         <v>150</v>
       </c>
-      <c r="E71" s="10" t="s">
+      <c r="E71" t="s">
         <v>270</v>
       </c>
-      <c r="F71" s="6">
+      <c r="F71">
         <v>27</v>
       </c>
       <c r="G71" t="s">
@@ -2848,10 +2863,10 @@
       <c r="D72" t="s">
         <v>152</v>
       </c>
-      <c r="E72" s="10" t="s">
+      <c r="E72" t="s">
         <v>284</v>
       </c>
-      <c r="F72" s="6">
+      <c r="F72">
         <v>0.29399999999999998</v>
       </c>
       <c r="G72" t="s">
@@ -2871,10 +2886,10 @@
       <c r="D73" t="s">
         <v>154</v>
       </c>
-      <c r="E73" s="10" t="s">
+      <c r="E73" t="s">
         <v>244</v>
       </c>
-      <c r="F73" s="6">
+      <c r="F73">
         <v>1.24</v>
       </c>
       <c r="G73" t="s">
@@ -2894,13 +2909,13 @@
       <c r="D74" t="s">
         <v>156</v>
       </c>
-      <c r="E74" s="11" t="s">
+      <c r="E74" s="7" t="s">
         <v>271</v>
       </c>
-      <c r="F74" s="12">
+      <c r="F74" s="7">
         <v>45</v>
       </c>
-      <c r="G74" s="11" t="s">
+      <c r="G74" s="9" t="s">
         <v>286</v>
       </c>
     </row>
@@ -2917,10 +2932,10 @@
       <c r="D75" t="s">
         <v>158</v>
       </c>
-      <c r="E75" s="10" t="s">
+      <c r="E75" t="s">
         <v>249</v>
       </c>
-      <c r="F75" s="6">
+      <c r="F75">
         <v>16.7</v>
       </c>
       <c r="G75" t="s">
@@ -2940,10 +2955,10 @@
       <c r="D76" t="s">
         <v>160</v>
       </c>
-      <c r="E76" s="10" t="s">
+      <c r="E76" t="s">
         <v>272</v>
       </c>
-      <c r="F76" s="6">
+      <c r="F76">
         <v>5.62</v>
       </c>
       <c r="G76" t="s">
@@ -2963,10 +2978,10 @@
       <c r="D77" t="s">
         <v>162</v>
       </c>
-      <c r="E77" s="10" t="s">
+      <c r="E77" t="s">
         <v>273</v>
       </c>
-      <c r="F77" s="9">
+      <c r="F77" s="6">
         <v>118000</v>
       </c>
       <c r="G77" t="s">
@@ -2986,7 +3001,7 @@
       <c r="D78" t="s">
         <v>164</v>
       </c>
-      <c r="G78" s="6" t="s">
+      <c r="G78" t="s">
         <v>195</v>
       </c>
     </row>
@@ -3003,7 +3018,7 @@
       <c r="D79" t="s">
         <v>166</v>
       </c>
-      <c r="G79" s="6" t="s">
+      <c r="G79" t="s">
         <v>195</v>
       </c>
     </row>
@@ -3023,7 +3038,7 @@
       <c r="E80" t="s">
         <v>290</v>
       </c>
-      <c r="F80" s="6">
+      <c r="F80">
         <v>49.5</v>
       </c>
       <c r="G80" t="s">
@@ -3043,7 +3058,7 @@
       <c r="D81" t="s">
         <v>172</v>
       </c>
-      <c r="G81" s="6" t="s">
+      <c r="G81" t="s">
         <v>195</v>
       </c>
     </row>
@@ -3060,7 +3075,7 @@
       <c r="D82" t="s">
         <v>175</v>
       </c>
-      <c r="G82" s="6" t="s">
+      <c r="G82" t="s">
         <v>195</v>
       </c>
     </row>
@@ -3077,7 +3092,7 @@
       <c r="D83" t="s">
         <v>178</v>
       </c>
-      <c r="G83" s="6" t="s">
+      <c r="G83" t="s">
         <v>195</v>
       </c>
     </row>
@@ -3097,7 +3112,7 @@
       <c r="E84" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="F84" s="7">
+      <c r="F84" s="3">
         <v>8.6900000000000005E-2</v>
       </c>
       <c r="G84" s="3" t="s">
@@ -3127,6 +3142,8 @@
     <hyperlink ref="G6" r:id="rId5" xr:uid="{80AC76BE-D6C1-494A-B6A4-50B84FF949CA}"/>
     <hyperlink ref="G10" r:id="rId6" xr:uid="{4DD938DE-8948-47A8-8630-85DF0C972A5C}"/>
     <hyperlink ref="G44" r:id="rId7" xr:uid="{523F7310-806C-481A-85FF-51B7F8B8EAAB}"/>
+    <hyperlink ref="G9" r:id="rId8" xr:uid="{FBACBB21-1F5D-43E9-901F-3651F9F72D65}"/>
+    <hyperlink ref="G74" r:id="rId9" location=":~:text=Currently%2C%20niobium%20prices%20range%20from,specialised%20products%20realise%20higher%20prices." xr:uid="{611CE029-EF7F-449F-AF7D-ADEC470297CE}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
start with production workflow
</commit_message>
<xml_diff>
--- a/data/manual/materials_prices.xlsx
+++ b/data/manual/materials_prices.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dpsich-my.sharepoint.com/personal/alvaro_hahn-menacho_psi_ch/Documents/Severin's work/3_Code/semesterproject/data/manual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="138" documentId="13_ncr:1_{D88AC83D-3D0E-48F6-B25A-3A931C8EAFD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31949691-E44D-420F-BA4F-560A928C2BB4}"/>
+  <xr:revisionPtr revIDLastSave="157" documentId="13_ncr:1_{D88AC83D-3D0E-48F6-B25A-3A931C8EAFD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AEFF2073-927D-408B-B424-8FF6646D1DC0}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="294">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="481" uniqueCount="297">
   <si>
     <t>material_category</t>
   </si>
@@ -915,6 +915,15 @@
   </si>
   <si>
     <t>https://ecoquery.ecoinvent.org/3.11/cutoff/dataset/2695/exchanges</t>
+  </si>
+  <si>
+    <t>https://github.com/polca/premise/blob/master/premise/data/additional_inventories/lci-PGM.xlsx</t>
+  </si>
+  <si>
+    <t>conversion factor dollar -&gt; Euro = 0.86</t>
+  </si>
+  <si>
+    <t>Average of platinum, palladium, rhodium, ruthenium, iridium</t>
   </si>
 </sst>
 </file>
@@ -961,7 +970,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
+        <fgColor theme="5" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -979,7 +988,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -990,10 +999,11 @@
     <xf numFmtId="11" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1299,7 +1309,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H84"/>
+  <dimension ref="A1:Q84"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
@@ -1535,16 +1545,16 @@
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="8" t="s">
+      <c r="B11" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="D11" s="10" t="s">
         <v>25</v>
       </c>
       <c r="E11" t="s">
@@ -1558,10 +1568,10 @@
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
       <c r="E12" t="s">
         <v>199</v>
       </c>
@@ -1911,16 +1921,16 @@
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="8" t="s">
+      <c r="A29" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B29" s="8" t="s">
+      <c r="B29" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="D29" s="8" t="s">
+      <c r="D29" s="10" t="s">
         <v>65</v>
       </c>
       <c r="E29" t="s">
@@ -1934,10 +1944,10 @@
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" s="8"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
+      <c r="A30" s="10"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="10"/>
+      <c r="D30" s="10"/>
       <c r="E30" t="s">
         <v>231</v>
       </c>
@@ -2583,16 +2593,16 @@
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A60" s="8" t="s">
+      <c r="A60" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="B60" s="8" t="s">
+      <c r="B60" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="C60" s="8" t="s">
+      <c r="C60" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="D60" s="8" t="s">
+      <c r="D60" s="10" t="s">
         <v>129</v>
       </c>
       <c r="E60" t="s">
@@ -2606,10 +2616,10 @@
       </c>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="8"/>
-      <c r="B61" s="8"/>
-      <c r="C61" s="8"/>
-      <c r="D61" s="8"/>
+      <c r="A61" s="10"/>
+      <c r="B61" s="10"/>
+      <c r="C61" s="10"/>
+      <c r="D61" s="10"/>
       <c r="E61" t="s">
         <v>205</v>
       </c>
@@ -2689,7 +2699,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>118</v>
       </c>
@@ -2712,7 +2722,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>118</v>
       </c>
@@ -2735,7 +2745,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>118</v>
       </c>
@@ -2758,7 +2768,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>118</v>
       </c>
@@ -2781,7 +2791,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>118</v>
       </c>
@@ -2804,7 +2814,7 @@
         <v>281</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>118</v>
       </c>
@@ -2827,7 +2837,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>118</v>
       </c>
@@ -2850,7 +2860,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>118</v>
       </c>
@@ -2873,7 +2883,7 @@
         <v>285</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>118</v>
       </c>
@@ -2896,7 +2906,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>118</v>
       </c>
@@ -2919,7 +2929,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>118</v>
       </c>
@@ -2942,7 +2952,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>118</v>
       </c>
@@ -2965,7 +2975,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>118</v>
       </c>
@@ -2988,7 +2998,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>118</v>
       </c>
@@ -3001,11 +3011,21 @@
       <c r="D78" t="s">
         <v>164</v>
       </c>
-      <c r="G78" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E78" s="7" t="s">
+        <v>164</v>
+      </c>
+      <c r="F78" s="7">
+        <f>107000*0.86</f>
+        <v>92020</v>
+      </c>
+      <c r="G78" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="Q78" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="79" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>118</v>
       </c>
@@ -3018,11 +3038,21 @@
       <c r="D79" t="s">
         <v>166</v>
       </c>
-      <c r="G79" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E79" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="F79" s="7">
+        <f>10300*0.86</f>
+        <v>8858</v>
+      </c>
+      <c r="G79" s="7" t="s">
+        <v>294</v>
+      </c>
+      <c r="Q79" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="80" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>118</v>
       </c>
@@ -3092,8 +3122,15 @@
       <c r="D83" t="s">
         <v>178</v>
       </c>
-      <c r="G83" t="s">
-        <v>195</v>
+      <c r="E83" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="F83" s="8">
+        <f>AVERAGE(F78:F79,F68:F69,F77)</f>
+        <v>54375.6</v>
+      </c>
+      <c r="G83" s="7" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.25">

</xml_diff>